<commit_message>
chore: aplicar limpeza segura da etapa 1 no GED_PROFISSIONAL
</commit_message>
<xml_diff>
--- a/scripts e caminhos das pastas.xlsx
+++ b/scripts e caminhos das pastas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0B4A23-FF50-45AD-9A2B-D2EB51BFF677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883AA8CC-5505-4986-A716-87DC5652B219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2610" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{82BB3B5E-D9B0-4AD5-AE42-8553B93553F4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{82BB3B5E-D9B0-4AD5-AE42-8553B93553F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -1991,7 +1991,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="59" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>142</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="123" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>190</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="143" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>39</v>
       </c>
@@ -2681,22 +2681,22 @@
         <v>211</v>
       </c>
     </row>
-    <row r="187" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="188" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="189" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>213</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>88</v>
       </c>
@@ -2950,9 +2950,12 @@
   <autoFilter ref="A1:A239" xr:uid="{D0608054-7E8C-4EEA-A390-DB7E9A50D952}">
     <filterColumn colId="0">
       <filters>
-        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\apps\documentos\templates\documentos\medicao.html"/>
-        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\media\documentos\versoes\I-ET-4880.00-9311-000-CZ1-001_RA.pdf"/>
-        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\media\healthcheck\test.txt"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\apps\documentos\static\documentos\logo_dorange.png"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\static\img\logo.png"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\static\videos\logo.png"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\staticfiles\documentos\logo_dorange.png"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\staticfiles\img\logo.png"/>
+        <filter val="C:\Users\daniel.laranjo\Documents\GED_PROFISSIONAL\staticfiles\videos\logo.png"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>